<commit_message>
Scrum: tablero al 27/10 (ClienteHttp hecho por Fernando) y guías actualizadas
- T-240 (HT-04) Done por Fernando; conexión de obra, semanas y proveedores Done; login web en Doing
- Registro del Sprint: 2 incidencias y 2 actividades del 27/10, fechas y evidencia de lo hecho hoy
- equipo/*.md con las tareas que quedan a cada uno

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtGmXDVgEBa1Hp6paBTjbG
</commit_message>
<xml_diff>
--- a/docs/scrum/SIGRO - Sprint 1 · Registro del Sprint.xlsx
+++ b/docs/scrum/SIGRO - Sprint 1 · Registro del Sprint.xlsx
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H30"/>
+  <dimension ref="B2:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1423,23 +1423,79 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
+    <row r="25" ht="44" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>El ClienteHttp (HT-04) bloqueaba la conexión de las pantallas web y seguía sin empezar a un día de la Review</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Fernando Istaña</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Scrum Master / Developer (web)</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>HT-04 · T-240</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Fernando lo programó y conectó obra, semanas y proveedores; Henry sigue con login, usuarios, roles y la conexión de almacén y costo</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Commit 27d66cc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>La API no guarda el código del presupuesto del S10 ni los días de entrega del proveedor, y no tiene endpoints de catálogo</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Víctor Adiel Luján</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Product Owner / backend</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>api/ (obra, compras, catálogo)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Pedido a Adiel: columna presupuesto en proyecto, dias_entrega en proveedor y endpoints del catálogo; compras sigue simulada hasta entonces</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>web/LEEME.md</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="6" t="n"/>
@@ -1476,6 +1532,24 @@
       <c r="F30" s="6" t="n"/>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1496,7 +1570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B3:H42"/>
+  <dimension ref="B3:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2178,23 +2252,75 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
+    <row r="26" ht="38" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Día 13</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Fernando Istaña</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Scrum Master</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Excel único de registro del sprint (incidencias, bitácora, tablero To Do/Doing/Done con criterios) y guías vigentes del equipo; ramas subidas a GitHub</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>T-253</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Día 13</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Fernando Istaña</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Developer (web)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>ClienteHttp: la web conectada a la API de Adiel (sesión, obras, semanas y proveedores) y pantalla mínima de ingreso; probado de punta a punta con PostgreSQL (commit 27d66cc)</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>T-240</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="6" t="n"/>
@@ -2313,8 +2439,26 @@
       <c r="G40" s="6" t="n"/>
       <c r="H40" s="6" t="n"/>
     </row>
+    <row r="41">
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+    </row>
     <row r="42">
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>Horas tomadas de los commits del repositorio; donde está vacía la completa el colaborador. Del 23/10 en adelante, una fila por actividad: fecha · hora · colaborador · qué hizo · T-xxx.</t>
         </is>
@@ -3040,26 +3184,42 @@
           <t>26/10</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
-        <is>
-          <t>T-004, T-006, T-240</t>
-        </is>
-      </c>
+      <c r="J12" s="12" t="n"/>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L12" s="12" t="n"/>
-      <c r="M12" s="12" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
       <c r="N12" s="13" t="inlineStr">
         <is>
           <t>La pantalla muestra los datos reales del servidor y sus errores</t>
         </is>
       </c>
-      <c r="O12" s="12" t="n"/>
-      <c r="P12" s="12" t="n"/>
-      <c r="Q12" s="13" t="n"/>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P12" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t>Commit 27d66cc (27/10), rama fernando-sprint1-web-integraciones</t>
+        </is>
+      </c>
       <c r="R12" s="12">
         <f>IF(AND(K12&lt;&gt;"To Do",L12&lt;&gt;"Sí"),"⚠ pasó a Doing sin DoR",IF(AND(K12="Done",O12&lt;&gt;"Sí"),"⚠ Done sin criterio cumplido",IF(AND(K12="Doing",COUNTIFS($G$6:$G$266,G12,$K$6:$K$266,"Doing",$E$6:$E$266,"&lt;&gt;Scrum")&gt;2,E12&lt;&gt;"Scrum"),"⚠ más de 2 en Doing","ok")))</f>
         <v/>
@@ -3712,26 +3872,42 @@
           <t>26/10</t>
         </is>
       </c>
-      <c r="J20" s="12" t="inlineStr">
-        <is>
-          <t>T-013, T-014, T-240</t>
-        </is>
-      </c>
+      <c r="J20" s="12" t="n"/>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L20" s="12" t="n"/>
-      <c r="M20" s="12" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
       <c r="N20" s="13" t="inlineStr">
         <is>
           <t>La pantalla muestra los datos reales del servidor y sus errores</t>
         </is>
       </c>
-      <c r="O20" s="12" t="n"/>
-      <c r="P20" s="12" t="n"/>
-      <c r="Q20" s="13" t="n"/>
+      <c r="O20" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P20" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Commit 27d66cc (27/10), rama fernando-sprint1-web-integraciones</t>
+        </is>
+      </c>
       <c r="R20" s="12">
         <f>IF(AND(K20&lt;&gt;"To Do",L20&lt;&gt;"Sí"),"⚠ pasó a Doing sin DoR",IF(AND(K20="Done",O20&lt;&gt;"Sí"),"⚠ Done sin criterio cumplido",IF(AND(K20="Doing",COUNTIFS($G$6:$G$266,G20,$K$6:$K$266,"Doing",$E$6:$E$266,"&lt;&gt;Scrum")&gt;2,E20&lt;&gt;"Scrum"),"⚠ más de 2 en Doing","ok")))</f>
         <v/>
@@ -5687,11 +5863,19 @@
       </c>
       <c r="K44" s="12" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L44" s="12" t="n"/>
-      <c r="M44" s="12" t="n"/>
+          <t>Doing</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
       <c r="N44" s="13" t="inlineStr">
         <is>
           <t>PR fusionado, build sin errores, modo claro/oscuro y escala 125 %</t>
@@ -5699,7 +5883,11 @@
       </c>
       <c r="O44" s="12" t="n"/>
       <c r="P44" s="12" t="n"/>
-      <c r="Q44" s="13" t="n"/>
+      <c r="Q44" s="13" t="inlineStr">
+        <is>
+          <t>Lienzo del Sprint 1</t>
+        </is>
+      </c>
       <c r="R44" s="12">
         <f>IF(AND(K44&lt;&gt;"To Do",L44&lt;&gt;"Sí"),"⚠ pasó a Doing sin DoR",IF(AND(K44="Done",O44&lt;&gt;"Sí"),"⚠ Done sin criterio cumplido",IF(AND(K44="Doing",COUNTIFS($G$6:$G$266,G44,$K$6:$K$266,"Doing",$E$6:$E$266,"&lt;&gt;Scrum")&gt;2,E44&lt;&gt;"Scrum"),"⚠ más de 2 en Doing","ok")))</f>
         <v/>
@@ -12873,7 +13061,7 @@
       </c>
       <c r="G134" s="12" t="inlineStr">
         <is>
-          <t>Henry</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="H134" s="12" t="n">
@@ -13225,7 +13413,7 @@
       </c>
       <c r="G138" s="12" t="inlineStr">
         <is>
-          <t>Henry</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="H138" s="12" t="n">
@@ -13236,26 +13424,42 @@
           <t>26/10</t>
         </is>
       </c>
-      <c r="J138" s="12" t="inlineStr">
-        <is>
-          <t>T-131, T-132, T-240</t>
-        </is>
-      </c>
+      <c r="J138" s="12" t="n"/>
       <c r="K138" s="12" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L138" s="12" t="n"/>
-      <c r="M138" s="12" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L138" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M138" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
       <c r="N138" s="13" t="inlineStr">
         <is>
           <t>La pantalla muestra los datos reales del servidor y sus errores</t>
         </is>
       </c>
-      <c r="O138" s="12" t="n"/>
-      <c r="P138" s="12" t="n"/>
-      <c r="Q138" s="13" t="n"/>
+      <c r="O138" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P138" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="Q138" s="13" t="inlineStr">
+        <is>
+          <t>Commit 27d66cc (27/10), rama fernando-sprint1-web-integraciones</t>
+        </is>
+      </c>
       <c r="R138" s="12">
         <f>IF(AND(K138&lt;&gt;"To Do",L138&lt;&gt;"Sí"),"⚠ pasó a Doing sin DoR",IF(AND(K138="Done",O138&lt;&gt;"Sí"),"⚠ Done sin criterio cumplido",IF(AND(K138="Doing",COUNTIFS($G$6:$G$266,G138,$K$6:$K$266,"Doing",$E$6:$E$266,"&lt;&gt;Scrum")&gt;2,E138&lt;&gt;"Scrum"),"⚠ más de 2 en Doing","ok")))</f>
         <v/>
@@ -13301,7 +13505,7 @@
       </c>
       <c r="G139" s="12" t="inlineStr">
         <is>
-          <t>Fernando</t>
+          <t>Henry</t>
         </is>
       </c>
       <c r="H139" s="12" t="n">
@@ -13545,7 +13749,7 @@
       </c>
       <c r="G142" s="12" t="inlineStr">
         <is>
-          <t>Henry</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="H142" s="12" t="n">
@@ -13897,7 +14101,7 @@
       </c>
       <c r="G146" s="12" t="inlineStr">
         <is>
-          <t>Henry</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="H146" s="12" t="n">
@@ -13908,26 +14112,42 @@
           <t>26/10</t>
         </is>
       </c>
-      <c r="J146" s="12" t="inlineStr">
-        <is>
-          <t>T-139, T-140, T-240</t>
-        </is>
-      </c>
+      <c r="J146" s="12" t="n"/>
       <c r="K146" s="12" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L146" s="12" t="n"/>
-      <c r="M146" s="12" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L146" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M146" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
       <c r="N146" s="13" t="inlineStr">
         <is>
           <t>La pantalla muestra los datos reales del servidor y sus errores</t>
         </is>
       </c>
-      <c r="O146" s="12" t="n"/>
-      <c r="P146" s="12" t="n"/>
-      <c r="Q146" s="13" t="n"/>
+      <c r="O146" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P146" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="Q146" s="13" t="inlineStr">
+        <is>
+          <t>Commit 27d66cc (27/10), rama fernando-sprint1-web-integraciones</t>
+        </is>
+      </c>
       <c r="R146" s="12">
         <f>IF(AND(K146&lt;&gt;"To Do",L146&lt;&gt;"Sí"),"⚠ pasó a Doing sin DoR",IF(AND(K146="Done",O146&lt;&gt;"Sí"),"⚠ Done sin criterio cumplido",IF(AND(K146="Doing",COUNTIFS($G$6:$G$266,G146,$K$6:$K$266,"Doing",$E$6:$E$266,"&lt;&gt;Scrum")&gt;2,E146&lt;&gt;"Scrum"),"⚠ más de 2 en Doing","ok")))</f>
         <v/>
@@ -13973,7 +14193,7 @@
       </c>
       <c r="G147" s="12" t="inlineStr">
         <is>
-          <t>Fernando</t>
+          <t>Henry</t>
         </is>
       </c>
       <c r="H147" s="12" t="n">
@@ -21857,7 +22077,7 @@
       </c>
       <c r="G245" s="12" t="inlineStr">
         <is>
-          <t>Henry</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="H245" s="12" t="n">
@@ -21871,19 +22091,39 @@
       <c r="J245" s="12" t="n"/>
       <c r="K245" s="12" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="L245" s="12" t="n"/>
-      <c r="M245" s="12" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L245" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M245" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
       <c r="N245" s="13" t="inlineStr">
         <is>
           <t>Entregable revisado por el equipo</t>
         </is>
       </c>
-      <c r="O245" s="12" t="n"/>
-      <c r="P245" s="12" t="n"/>
-      <c r="Q245" s="13" t="n"/>
+      <c r="O245" s="12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P245" s="12" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="Q245" s="13" t="inlineStr">
+        <is>
+          <t>Commit 27d66cc (27/10), rama fernando-sprint1-web-integraciones</t>
+        </is>
+      </c>
       <c r="R245" s="12">
         <f>IF(AND(K245&lt;&gt;"To Do",L245&lt;&gt;"Sí"),"⚠ pasó a Doing sin DoR",IF(AND(K245="Done",O245&lt;&gt;"Sí"),"⚠ Done sin criterio cumplido",IF(AND(K245="Doing",COUNTIFS($G$6:$G$266,G245,$K$6:$K$266,"Doing",$E$6:$E$266,"&lt;&gt;Scrum")&gt;2,E245&lt;&gt;"Scrum"),"⚠ más de 2 en Doing","ok")))</f>
         <v/>
@@ -32572,7 +32812,7 @@
       </c>
       <c r="F12" s="35" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-004, T-006, T-240. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Estado: Done — commit 27d66cc: crea la obra en el servidor. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -32728,7 +32968,7 @@
       </c>
       <c r="F20" s="35" t="inlineStr">
         <is>
-          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-013, T-014, T-240. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Estado: Done — commit 27d66cc: semanas desde /obras/{id}/periodos. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -33196,7 +33436,7 @@
       </c>
       <c r="F44" s="35" t="inlineStr">
         <is>
-          <t>Henry programa la pantalla en web/ (React + TypeScript + CSS) según la pantalla 1 (app) y 20 (web) · Login, con los componentes del sistema de diseño, modo claro y oscuro, y escala de texto; la web no calcula saldos ni costos. Empieza después de T-035. 3 h · límite 26/10.</t>
+          <t>Henry programa la pantalla en web/ (React + TypeScript + CSS) según la pantalla 1 (app) y 20 (web) · Login, con los componentes del sistema de diseño, modo claro y oscuro, y escala de texto; la web no calcula saldos ni costos. Estado: Doing — versión mínima y sesión hechas (27d66cc); falta la pantalla 20 del lienzo. Empieza después de T-035. 3 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -34962,7 +35202,7 @@
       </c>
       <c r="F134" s="35" t="inlineStr">
         <is>
-          <t>Henry dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Empieza después de T-128. 1 h · límite 24/10.</t>
+          <t>Fernando dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Empieza después de T-128. 1 h · límite 24/10.</t>
         </is>
       </c>
     </row>
@@ -35038,7 +35278,7 @@
       </c>
       <c r="F138" s="35" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-131, T-132, T-240. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Estado: Done — commit 27d66cc: 626 proveedores desde la API. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -35057,7 +35297,7 @@
       </c>
       <c r="F139" s="35" t="inlineStr">
         <is>
-          <t>Fernando, que no programó lo que falta de HU-29, prueba los endpoints con Postman y la interfaz contra cada condición final de la tarjeta 3 en el ambiente de pruebas; si todo cumple aprueba el PR, si no lo devuelve con la falla. Estado: To Do — alguien distinto del autor (T1, T5, T8). Empieza después de T-130, T-131, T-132, T-133, T-233. 1 h · límite 27/10.</t>
+          <t>Henry, que no programó lo que falta de HU-29, prueba los endpoints con Postman y la interfaz contra cada condición final de la tarjeta 3 en el ambiente de pruebas; si todo cumple aprueba el PR, si no lo devuelve con la falla. Estado: To Do — alguien distinto del autor (T1, T5, T8). Empieza después de T-130, T-131, T-132, T-133, T-233. 1 h · límite 27/10.</t>
         </is>
       </c>
     </row>
@@ -35118,7 +35358,7 @@
       </c>
       <c r="F142" s="35" t="inlineStr">
         <is>
-          <t>Henry dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Empieza después de T-136. 1 h · límite 24/10.</t>
+          <t>Fernando dibuja el diagrama UML que explica cómo funciona la HU (actores, pantallas, API y base) para que quien programa no tenga que adivinar el flujo. Empieza después de T-136. 1 h · límite 24/10.</t>
         </is>
       </c>
     </row>
@@ -35194,7 +35434,7 @@
       </c>
       <c r="F146" s="35" t="inlineStr">
         <is>
-          <t>Henry cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Empieza después de T-139, T-140, T-240. 2 h · límite 26/10.</t>
+          <t>Fernando cambia los datos simulados por la API real a través del ClienteHttp: la pantalla muestra lo que devuelve el servidor y sus errores {codigo, mensaje}. Estado: Done — commit 27d66cc: RUC duplicado rechazado por el servidor. 2 h · límite 26/10.</t>
         </is>
       </c>
     </row>
@@ -35213,7 +35453,7 @@
       </c>
       <c r="F147" s="35" t="inlineStr">
         <is>
-          <t>Fernando, que no programó lo que falta de HU-30, prueba los endpoints con Postman y la interfaz contra cada condición final de la tarjeta 3 en el ambiente de pruebas; si todo cumple aprueba el PR, si no lo devuelve con la falla. Estado: To Do — alguien distinto del autor (T1, T5, T8). Empieza después de T-138, T-139, T-140, T-141, T-233. 1 h · límite 27/10.</t>
+          <t>Henry, que no programó lo que falta de HU-30, prueba los endpoints con Postman y la interfaz contra cada condición final de la tarjeta 3 en el ambiente de pruebas; si todo cumple aprueba el PR, si no lo devuelve con la falla. Estado: To Do — alguien distinto del autor (T1, T5, T8). Empieza después de T-138, T-139, T-140, T-141, T-233. 1 h · límite 27/10.</t>
         </is>
       </c>
     </row>
@@ -37151,7 +37391,7 @@
       </c>
       <c r="F245" s="35" t="inlineStr">
         <is>
-          <t>Henry: Habilitador de la web: una sola pieza que usan todas las pantallas para hablar con la API. Estado: To Do — desbloquea todas las tareas «Conectar…». 4 h · límite 26/10.</t>
+          <t>Fernando: Habilitador de la web: una sola pieza que usan todas las pantallas para hablar con la API. Estado: Done — commit 27d66cc (27/10); lo tomó Fernando para destrabar la conexión. 4 h · límite 26/10.</t>
         </is>
       </c>
     </row>

</xml_diff>